<commit_message>
updated data sheet with URLs from 5 pages
</commit_message>
<xml_diff>
--- a/DataSheet/RiskPrediction2017.xlsx
+++ b/DataSheet/RiskPrediction2017.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="45" windowWidth="20115" windowHeight="7995" firstSheet="2" activeTab="8"/>
+    <workbookView xWindow="240" yWindow="45" windowWidth="20115" windowHeight="7995" firstSheet="2" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Mandatory Keywords" sheetId="4" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="767">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="772">
   <si>
     <t>Keywords</t>
   </si>
@@ -1681,9 +1681,6 @@
     <t>Google search engine - APIs</t>
   </si>
   <si>
-    <t xml:space="preserve">Bing serach engine - APIs </t>
-  </si>
-  <si>
     <t>1st page</t>
   </si>
   <si>
@@ -2327,13 +2324,31 @@
   </si>
   <si>
     <t>google.co.zw</t>
+  </si>
+  <si>
+    <t>Google URLs for first 5 pages</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=dsk+developers+ltd&amp;oq=dsk+developers+ltd&amp;aqs=chrome..69i57.10393j0j7&amp;sourceid=chrome&amp;ie=UTF-8</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=dsk+developers+ltd&amp;sxsrf=ACYBGNQn-2TC1rAjySPaEqfmbT0PYP_TaA:1581828616895&amp;ei=CMpIXuGkNvHjz7sPhq6Y6AU&amp;start=10&amp;sa=N&amp;ved=2ahUKEwjhyLjmotXnAhXx8XMBHQYXBl0Q8tMDegQIDhAu&amp;cshid=1581828673698172&amp;biw=1366&amp;bih=387</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=dsk+developers+ltd&amp;sxsrf=ACYBGNTtgcWrGj00rldhaNMwjlMkoriRxQ:1581957064648&amp;ei=yL9KXuKhJ-bcz7sP3LCRoAQ&amp;start=20&amp;sa=N&amp;ved=2ahUKEwjipY2ngdnnAhVm7nMBHVxYBEQ4ChDy0wN6BAgMEDA&amp;biw=1366&amp;bih=375</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=dsk+developers+ltd&amp;sxsrf=ACYBGNSXZgtKy6RrFnIACekhKSmQsxeviw:1581957100366&amp;ei=7L9KXqb7FcbDz7sPreyTmAE&amp;start=30&amp;sa=N&amp;ved=2ahUKEwimoZG4gdnnAhXG4XMBHS32BBM4FBDy0wN6BAgMEDI&amp;biw=1366&amp;bih=370</t>
+  </si>
+  <si>
+    <t>https://www.google.com/search?q=dsk+developers+ltd&amp;sxsrf=ACYBGNRxl_DGZu6K2Z22RgMmqy-4GTETEA:1581957260480&amp;ei=jMBKXtH5HN3Wz7sP4rK5uAE&amp;start=40&amp;sa=N&amp;ved=2ahUKEwjR772EgtnnAhVd63MBHWJZDhc4HhDy0wN6BAgMEDQ&amp;biw=1366&amp;bih=216</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2506,6 +2521,13 @@
       <color rgb="FF000000"/>
       <name val="Verdana"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF008080"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="35">
@@ -2880,7 +2902,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1" applyProtection="1"/>
@@ -2896,15 +2918,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="10" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3249,10 +3272,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="42.75" customHeight="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="13"/>
+      <c r="B1" s="15"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
@@ -3349,10 +3372,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="46.5" customHeight="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="13"/>
+      <c r="B1" s="15"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
@@ -6652,7 +6675,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>547</v>
@@ -6665,7 +6688,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>549</v>
@@ -6673,38 +6696,56 @@
     </row>
     <row r="6" spans="1:4">
       <c r="B6" s="7" t="s">
-        <v>551</v>
+        <v>766</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9">
         <v>1</v>
       </c>
+      <c r="B9" s="16" t="s">
+        <v>767</v>
+      </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10">
         <v>2</v>
       </c>
+      <c r="B10" s="16" t="s">
+        <v>768</v>
+      </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11">
         <v>3</v>
       </c>
+      <c r="B11" s="2" t="s">
+        <v>769</v>
+      </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12">
         <v>4</v>
       </c>
+      <c r="B12" s="2" t="s">
+        <v>770</v>
+      </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13">
         <v>5</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>771</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1"/>
     <hyperlink ref="B3" r:id="rId2"/>
+    <hyperlink ref="B11" r:id="rId3"/>
+    <hyperlink ref="B12" r:id="rId4"/>
+    <hyperlink ref="B13" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6726,1034 +6767,1034 @@
   <sheetData>
     <row r="1" spans="1:10" s="7" customFormat="1">
       <c r="A1" s="7" t="s">
+        <v>553</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>554</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="7" t="s">
         <v>555</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>556</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>557</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>558</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>559</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>560</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="I1" s="7" t="s">
         <v>561</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>562</v>
       </c>
-      <c r="J1" s="7" t="s">
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="13" t="s">
         <v>563</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="14" t="s">
+      <c r="B2" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="13" t="s">
         <v>565</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="14" t="s">
+      <c r="B3" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="B3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="13" t="s">
         <v>567</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="14" t="s">
+      <c r="B4" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="13" t="s">
         <v>569</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="14" t="s">
+      <c r="B5" s="2" t="s">
         <v>570</v>
       </c>
-      <c r="B5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="13" t="s">
         <v>571</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="14" t="s">
+      <c r="B6" s="2" t="s">
         <v>572</v>
       </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="13" t="s">
         <v>573</v>
       </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="14" t="s">
+      <c r="B7" s="2" t="s">
         <v>574</v>
       </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="13" t="s">
         <v>575</v>
       </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="14" t="s">
+      <c r="B8" s="2" t="s">
         <v>576</v>
       </c>
-      <c r="B8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:10" ht="30">
+      <c r="A9" s="13" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="30">
-      <c r="A9" s="14" t="s">
+      <c r="B9" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="B9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="13" t="s">
         <v>579</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="14" t="s">
+      <c r="B10" s="2" t="s">
         <v>580</v>
       </c>
-      <c r="B10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="13" t="s">
         <v>581</v>
       </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="14" t="s">
+      <c r="B11" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="B11" s="2" t="s">
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="13" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="14" t="s">
+    <row r="13" spans="1:10" ht="30">
+      <c r="A13" s="13" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30">
-      <c r="A13" s="14" t="s">
+    <row r="14" spans="1:10">
+      <c r="A14" s="13" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="14" t="s">
+    <row r="15" spans="1:10">
+      <c r="A15" s="13" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="14" t="s">
+    <row r="16" spans="1:10">
+      <c r="A16" s="13" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
-      <c r="A16" s="14" t="s">
+    <row r="17" spans="1:1" ht="30">
+      <c r="A17" s="13" t="s">
         <v>588</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="30">
-      <c r="A17" s="14" t="s">
+    <row r="18" spans="1:1" ht="30">
+      <c r="A18" s="13" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="30">
-      <c r="A18" s="14" t="s">
+    <row r="19" spans="1:1" ht="30">
+      <c r="A19" s="13" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="30">
-      <c r="A19" s="14" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" s="13" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="14" t="s">
+    <row r="21" spans="1:1" ht="30">
+      <c r="A21" s="13" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="30">
-      <c r="A21" s="14" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" s="13" t="s">
         <v>593</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
-      <c r="A22" s="14" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" s="13" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
-      <c r="A23" s="14" t="s">
+    <row r="24" spans="1:1" ht="30">
+      <c r="A24" s="13" t="s">
         <v>595</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="30">
-      <c r="A24" s="14" t="s">
+    <row r="25" spans="1:1">
+      <c r="A25" s="13" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
-      <c r="A25" s="14" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" s="13" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
-      <c r="A26" s="14" t="s">
+    <row r="27" spans="1:1" ht="30">
+      <c r="A27" s="13" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="30">
-      <c r="A27" s="14" t="s">
+    <row r="28" spans="1:1">
+      <c r="A28" s="13" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
-      <c r="A28" s="14" t="s">
+    <row r="29" spans="1:1" ht="30">
+      <c r="A29" s="13" t="s">
         <v>600</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="30">
-      <c r="A29" s="14" t="s">
+    <row r="30" spans="1:1">
+      <c r="A30" s="13" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
-      <c r="A30" s="14" t="s">
+    <row r="31" spans="1:1">
+      <c r="A31" s="13" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="31" spans="1:1">
-      <c r="A31" s="14" t="s">
+    <row r="32" spans="1:1">
+      <c r="A32" s="13" t="s">
         <v>603</v>
       </c>
     </row>
-    <row r="32" spans="1:1">
-      <c r="A32" s="14" t="s">
+    <row r="33" spans="1:1" ht="30">
+      <c r="A33" s="13" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="30">
-      <c r="A33" s="14" t="s">
+    <row r="34" spans="1:1">
+      <c r="A34" s="13" t="s">
         <v>605</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
-      <c r="A34" s="14" t="s">
+    <row r="35" spans="1:1">
+      <c r="A35" s="13" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
-      <c r="A35" s="14" t="s">
+    <row r="36" spans="1:1">
+      <c r="A36" s="13" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="36" spans="1:1">
-      <c r="A36" s="14" t="s">
+    <row r="37" spans="1:1">
+      <c r="A37" s="13" t="s">
         <v>608</v>
       </c>
     </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="14" t="s">
+    <row r="38" spans="1:1">
+      <c r="A38" s="13" t="s">
         <v>609</v>
       </c>
     </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="14" t="s">
+    <row r="39" spans="1:1">
+      <c r="A39" s="13" t="s">
         <v>610</v>
       </c>
     </row>
-    <row r="39" spans="1:1">
-      <c r="A39" s="14" t="s">
+    <row r="40" spans="1:1">
+      <c r="A40" s="13" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="40" spans="1:1">
-      <c r="A40" s="14" t="s">
+    <row r="41" spans="1:1">
+      <c r="A41" s="13" t="s">
         <v>612</v>
       </c>
     </row>
-    <row r="41" spans="1:1">
-      <c r="A41" s="14" t="s">
+    <row r="42" spans="1:1" ht="30">
+      <c r="A42" s="13" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="42" spans="1:1" ht="30">
-      <c r="A42" s="14" t="s">
+    <row r="43" spans="1:1">
+      <c r="A43" s="13" t="s">
         <v>614</v>
       </c>
     </row>
-    <row r="43" spans="1:1">
-      <c r="A43" s="14" t="s">
+    <row r="44" spans="1:1">
+      <c r="A44" s="13" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="44" spans="1:1">
-      <c r="A44" s="14" t="s">
+    <row r="45" spans="1:1">
+      <c r="A45" s="13" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="14" t="s">
+    <row r="46" spans="1:1" ht="30">
+      <c r="A46" s="14" t="s">
         <v>617</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="30">
-      <c r="A46" s="15" t="s">
+    <row r="47" spans="1:1">
+      <c r="A47" s="13" t="s">
         <v>618</v>
       </c>
     </row>
-    <row r="47" spans="1:1">
-      <c r="A47" s="14" t="s">
+    <row r="48" spans="1:1">
+      <c r="A48" s="13" t="s">
         <v>619</v>
       </c>
     </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="14" t="s">
+    <row r="49" spans="1:1" ht="30">
+      <c r="A49" s="13" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="30">
-      <c r="A49" s="14" t="s">
+    <row r="50" spans="1:1" ht="30">
+      <c r="A50" s="13" t="s">
         <v>621</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="30">
-      <c r="A50" s="14" t="s">
+    <row r="51" spans="1:1">
+      <c r="A51" s="13" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
-      <c r="A51" s="14" t="s">
+    <row r="52" spans="1:1">
+      <c r="A52" s="13" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="52" spans="1:1">
-      <c r="A52" s="14" t="s">
+    <row r="53" spans="1:1">
+      <c r="A53" s="13" t="s">
         <v>624</v>
       </c>
     </row>
-    <row r="53" spans="1:1">
-      <c r="A53" s="14" t="s">
+    <row r="54" spans="1:1">
+      <c r="A54" s="13" t="s">
         <v>625</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
-      <c r="A54" s="14" t="s">
+    <row r="55" spans="1:1" ht="30">
+      <c r="A55" s="13" t="s">
         <v>626</v>
       </c>
     </row>
-    <row r="55" spans="1:1" ht="30">
-      <c r="A55" s="14" t="s">
+    <row r="56" spans="1:1" ht="30">
+      <c r="A56" s="13" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="56" spans="1:1" ht="30">
-      <c r="A56" s="14" t="s">
+    <row r="57" spans="1:1" ht="30">
+      <c r="A57" s="13" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="57" spans="1:1" ht="30">
-      <c r="A57" s="14" t="s">
+    <row r="58" spans="1:1" ht="30">
+      <c r="A58" s="13" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="30">
-      <c r="A58" s="14" t="s">
+    <row r="59" spans="1:1">
+      <c r="A59" s="13" t="s">
         <v>630</v>
       </c>
     </row>
-    <row r="59" spans="1:1">
-      <c r="A59" s="14" t="s">
+    <row r="60" spans="1:1" ht="30">
+      <c r="A60" s="13" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="60" spans="1:1" ht="30">
-      <c r="A60" s="14" t="s">
+    <row r="61" spans="1:1">
+      <c r="A61" s="13" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="61" spans="1:1">
-      <c r="A61" s="14" t="s">
+    <row r="62" spans="1:1">
+      <c r="A62" s="13" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
-      <c r="A62" s="14" t="s">
+    <row r="63" spans="1:1">
+      <c r="A63" s="13" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
-      <c r="A63" s="14" t="s">
+    <row r="64" spans="1:1">
+      <c r="A64" s="13" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="64" spans="1:1">
-      <c r="A64" s="14" t="s">
+    <row r="65" spans="1:1">
+      <c r="A65" s="13" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="14" t="s">
+    <row r="66" spans="1:1">
+      <c r="A66" s="13" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="14" t="s">
+    <row r="67" spans="1:1">
+      <c r="A67" s="13" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="67" spans="1:1">
-      <c r="A67" s="14" t="s">
+    <row r="68" spans="1:1" ht="30">
+      <c r="A68" s="13" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="68" spans="1:1" ht="30">
-      <c r="A68" s="14" t="s">
+    <row r="69" spans="1:1">
+      <c r="A69" s="13" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="69" spans="1:1">
-      <c r="A69" s="14" t="s">
+    <row r="70" spans="1:1">
+      <c r="A70" s="13" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="70" spans="1:1">
-      <c r="A70" s="14" t="s">
+    <row r="71" spans="1:1">
+      <c r="A71" s="13" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="71" spans="1:1">
-      <c r="A71" s="14" t="s">
+    <row r="72" spans="1:1">
+      <c r="A72" s="13" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="72" spans="1:1">
-      <c r="A72" s="14" t="s">
+    <row r="73" spans="1:1">
+      <c r="A73" s="13" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="73" spans="1:1">
-      <c r="A73" s="14" t="s">
+    <row r="74" spans="1:1">
+      <c r="A74" s="13" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="74" spans="1:1">
-      <c r="A74" s="14" t="s">
+    <row r="75" spans="1:1">
+      <c r="A75" s="13" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="75" spans="1:1">
-      <c r="A75" s="14" t="s">
+    <row r="76" spans="1:1">
+      <c r="A76" s="13" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="76" spans="1:1">
-      <c r="A76" s="14" t="s">
+    <row r="77" spans="1:1">
+      <c r="A77" s="13" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="77" spans="1:1">
-      <c r="A77" s="14" t="s">
+    <row r="78" spans="1:1" ht="30">
+      <c r="A78" s="13" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="78" spans="1:1" ht="30">
-      <c r="A78" s="14" t="s">
+    <row r="79" spans="1:1">
+      <c r="A79" s="13" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="79" spans="1:1">
-      <c r="A79" s="14" t="s">
+    <row r="80" spans="1:1">
+      <c r="A80" s="13" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="80" spans="1:1">
-      <c r="A80" s="14" t="s">
+    <row r="81" spans="1:1">
+      <c r="A81" s="13" t="s">
         <v>652</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
-      <c r="A81" s="14" t="s">
+    <row r="82" spans="1:1">
+      <c r="A82" s="13" t="s">
         <v>653</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
-      <c r="A82" s="14" t="s">
+    <row r="83" spans="1:1">
+      <c r="A83" s="13" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="83" spans="1:1">
-      <c r="A83" s="14" t="s">
+    <row r="84" spans="1:1">
+      <c r="A84" s="13" t="s">
         <v>655</v>
       </c>
     </row>
-    <row r="84" spans="1:1">
-      <c r="A84" s="14" t="s">
+    <row r="85" spans="1:1">
+      <c r="A85" s="13" t="s">
         <v>656</v>
       </c>
     </row>
-    <row r="85" spans="1:1">
-      <c r="A85" s="14" t="s">
+    <row r="86" spans="1:1">
+      <c r="A86" s="13" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="86" spans="1:1">
-      <c r="A86" s="14" t="s">
+    <row r="87" spans="1:1">
+      <c r="A87" s="13" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="87" spans="1:1">
-      <c r="A87" s="14" t="s">
+    <row r="88" spans="1:1">
+      <c r="A88" s="13" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="30">
+      <c r="A89" s="13" t="s">
         <v>659</v>
       </c>
     </row>
-    <row r="88" spans="1:1">
-      <c r="A88" s="14" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" ht="30">
-      <c r="A89" s="14" t="s">
+    <row r="90" spans="1:1">
+      <c r="A90" s="13" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="90" spans="1:1">
-      <c r="A90" s="14" t="s">
+    <row r="91" spans="1:1">
+      <c r="A91" s="13" t="s">
         <v>661</v>
       </c>
     </row>
-    <row r="91" spans="1:1">
-      <c r="A91" s="14" t="s">
+    <row r="92" spans="1:1">
+      <c r="A92" s="13" t="s">
         <v>662</v>
       </c>
     </row>
-    <row r="92" spans="1:1">
-      <c r="A92" s="14" t="s">
+    <row r="93" spans="1:1">
+      <c r="A93" s="13" t="s">
         <v>663</v>
       </c>
     </row>
-    <row r="93" spans="1:1">
-      <c r="A93" s="14" t="s">
+    <row r="94" spans="1:1">
+      <c r="A94" s="13" t="s">
         <v>664</v>
       </c>
     </row>
-    <row r="94" spans="1:1">
-      <c r="A94" s="14" t="s">
+    <row r="95" spans="1:1">
+      <c r="A95" s="13" t="s">
         <v>665</v>
       </c>
     </row>
-    <row r="95" spans="1:1">
-      <c r="A95" s="14" t="s">
+    <row r="96" spans="1:1" ht="30">
+      <c r="A96" s="13" t="s">
         <v>666</v>
       </c>
     </row>
-    <row r="96" spans="1:1" ht="30">
-      <c r="A96" s="14" t="s">
+    <row r="97" spans="1:1" ht="30">
+      <c r="A97" s="13" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="97" spans="1:1" ht="30">
-      <c r="A97" s="14" t="s">
+    <row r="98" spans="1:1">
+      <c r="A98" s="13" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="98" spans="1:1">
-      <c r="A98" s="14" t="s">
+    <row r="99" spans="1:1">
+      <c r="A99" s="13" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="99" spans="1:1">
-      <c r="A99" s="14" t="s">
+    <row r="100" spans="1:1">
+      <c r="A100" s="13" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="100" spans="1:1">
-      <c r="A100" s="14" t="s">
+    <row r="101" spans="1:1">
+      <c r="A101" s="13" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="101" spans="1:1">
-      <c r="A101" s="14" t="s">
+    <row r="102" spans="1:1">
+      <c r="A102" s="13" t="s">
         <v>672</v>
       </c>
     </row>
-    <row r="102" spans="1:1">
-      <c r="A102" s="14" t="s">
+    <row r="103" spans="1:1">
+      <c r="A103" s="13" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="103" spans="1:1">
-      <c r="A103" s="14" t="s">
+    <row r="104" spans="1:1">
+      <c r="A104" s="13" t="s">
         <v>674</v>
       </c>
     </row>
-    <row r="104" spans="1:1">
-      <c r="A104" s="14" t="s">
+    <row r="105" spans="1:1">
+      <c r="A105" s="13" t="s">
         <v>675</v>
       </c>
     </row>
-    <row r="105" spans="1:1">
-      <c r="A105" s="14" t="s">
+    <row r="106" spans="1:1">
+      <c r="A106" s="13" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="106" spans="1:1">
-      <c r="A106" s="14" t="s">
+    <row r="107" spans="1:1">
+      <c r="A107" s="13" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="107" spans="1:1">
-      <c r="A107" s="14" t="s">
+    <row r="108" spans="1:1">
+      <c r="A108" s="13" t="s">
         <v>678</v>
       </c>
     </row>
-    <row r="108" spans="1:1">
-      <c r="A108" s="14" t="s">
+    <row r="109" spans="1:1" ht="30">
+      <c r="A109" s="13" t="s">
         <v>679</v>
       </c>
     </row>
-    <row r="109" spans="1:1" ht="30">
-      <c r="A109" s="14" t="s">
+    <row r="110" spans="1:1">
+      <c r="A110" s="13" t="s">
         <v>680</v>
       </c>
     </row>
-    <row r="110" spans="1:1">
-      <c r="A110" s="14" t="s">
+    <row r="111" spans="1:1">
+      <c r="A111" s="13" t="s">
         <v>681</v>
       </c>
     </row>
-    <row r="111" spans="1:1">
-      <c r="A111" s="14" t="s">
+    <row r="112" spans="1:1" ht="30">
+      <c r="A112" s="13" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="112" spans="1:1" ht="30">
-      <c r="A112" s="14" t="s">
+    <row r="113" spans="1:1">
+      <c r="A113" s="13" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="113" spans="1:1">
-      <c r="A113" s="14" t="s">
+    <row r="114" spans="1:1" ht="30">
+      <c r="A114" s="13" t="s">
         <v>684</v>
       </c>
     </row>
-    <row r="114" spans="1:1" ht="30">
-      <c r="A114" s="14" t="s">
+    <row r="115" spans="1:1">
+      <c r="A115" s="13" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="115" spans="1:1">
-      <c r="A115" s="14" t="s">
+    <row r="116" spans="1:1">
+      <c r="A116" s="13" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="116" spans="1:1">
-      <c r="A116" s="14" t="s">
+    <row r="117" spans="1:1">
+      <c r="A117" s="13" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="117" spans="1:1">
-      <c r="A117" s="14" t="s">
+    <row r="118" spans="1:1">
+      <c r="A118" s="13" t="s">
         <v>688</v>
       </c>
     </row>
-    <row r="118" spans="1:1">
-      <c r="A118" s="14" t="s">
+    <row r="119" spans="1:1">
+      <c r="A119" s="13" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="119" spans="1:1">
-      <c r="A119" s="14" t="s">
+    <row r="120" spans="1:1">
+      <c r="A120" s="13" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="120" spans="1:1">
-      <c r="A120" s="14" t="s">
+    <row r="121" spans="1:1">
+      <c r="A121" s="13" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="121" spans="1:1">
-      <c r="A121" s="14" t="s">
+    <row r="122" spans="1:1" ht="30">
+      <c r="A122" s="13" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="122" spans="1:1" ht="30">
-      <c r="A122" s="14" t="s">
+    <row r="123" spans="1:1">
+      <c r="A123" s="13" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="123" spans="1:1">
-      <c r="A123" s="14" t="s">
+    <row r="124" spans="1:1" ht="30">
+      <c r="A124" s="13" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="124" spans="1:1" ht="30">
-      <c r="A124" s="14" t="s">
+    <row r="125" spans="1:1">
+      <c r="A125" s="13" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="125" spans="1:1">
-      <c r="A125" s="14" t="s">
+    <row r="126" spans="1:1">
+      <c r="A126" s="13" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="126" spans="1:1">
-      <c r="A126" s="14" t="s">
+    <row r="127" spans="1:1">
+      <c r="A127" s="13" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="127" spans="1:1">
-      <c r="A127" s="14" t="s">
+    <row r="128" spans="1:1">
+      <c r="A128" s="13" t="s">
         <v>698</v>
       </c>
     </row>
-    <row r="128" spans="1:1">
-      <c r="A128" s="14" t="s">
+    <row r="129" spans="1:1" ht="30">
+      <c r="A129" s="13" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="129" spans="1:1" ht="30">
-      <c r="A129" s="14" t="s">
+    <row r="130" spans="1:1">
+      <c r="A130" s="13" t="s">
         <v>700</v>
       </c>
     </row>
-    <row r="130" spans="1:1">
-      <c r="A130" s="14" t="s">
+    <row r="131" spans="1:1" ht="30">
+      <c r="A131" s="13" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="131" spans="1:1" ht="30">
-      <c r="A131" s="14" t="s">
+    <row r="132" spans="1:1">
+      <c r="A132" s="13" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="132" spans="1:1">
-      <c r="A132" s="14" t="s">
+    <row r="133" spans="1:1" ht="30">
+      <c r="A133" s="13" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="133" spans="1:1" ht="30">
-      <c r="A133" s="14" t="s">
+    <row r="134" spans="1:1" ht="30">
+      <c r="A134" s="13" t="s">
         <v>704</v>
       </c>
     </row>
-    <row r="134" spans="1:1" ht="30">
-      <c r="A134" s="14" t="s">
+    <row r="135" spans="1:1">
+      <c r="A135" s="13" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="135" spans="1:1">
-      <c r="A135" s="14" t="s">
+    <row r="136" spans="1:1" ht="30">
+      <c r="A136" s="13" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="136" spans="1:1" ht="30">
-      <c r="A136" s="14" t="s">
+    <row r="137" spans="1:1" ht="30">
+      <c r="A137" s="13" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="137" spans="1:1" ht="30">
-      <c r="A137" s="14" t="s">
+    <row r="138" spans="1:1" ht="30">
+      <c r="A138" s="13" t="s">
         <v>708</v>
       </c>
     </row>
-    <row r="138" spans="1:1" ht="30">
-      <c r="A138" s="14" t="s">
+    <row r="139" spans="1:1" ht="30">
+      <c r="A139" s="13" t="s">
         <v>709</v>
       </c>
     </row>
-    <row r="139" spans="1:1" ht="30">
-      <c r="A139" s="14" t="s">
+    <row r="140" spans="1:1" ht="30">
+      <c r="A140" s="13" t="s">
         <v>710</v>
       </c>
     </row>
-    <row r="140" spans="1:1" ht="30">
-      <c r="A140" s="14" t="s">
+    <row r="141" spans="1:1">
+      <c r="A141" s="13" t="s">
         <v>711</v>
       </c>
     </row>
-    <row r="141" spans="1:1">
-      <c r="A141" s="14" t="s">
+    <row r="142" spans="1:1">
+      <c r="A142" s="13" t="s">
         <v>712</v>
       </c>
     </row>
-    <row r="142" spans="1:1">
-      <c r="A142" s="14" t="s">
+    <row r="143" spans="1:1">
+      <c r="A143" s="13" t="s">
         <v>713</v>
       </c>
     </row>
-    <row r="143" spans="1:1">
-      <c r="A143" s="14" t="s">
+    <row r="144" spans="1:1" ht="30">
+      <c r="A144" s="13" t="s">
         <v>714</v>
       </c>
     </row>
-    <row r="144" spans="1:1" ht="30">
-      <c r="A144" s="14" t="s">
+    <row r="145" spans="1:1" ht="30">
+      <c r="A145" s="13" t="s">
         <v>715</v>
       </c>
     </row>
-    <row r="145" spans="1:1" ht="30">
-      <c r="A145" s="14" t="s">
+    <row r="146" spans="1:1">
+      <c r="A146" s="13" t="s">
         <v>716</v>
       </c>
     </row>
-    <row r="146" spans="1:1">
-      <c r="A146" s="14" t="s">
+    <row r="147" spans="1:1">
+      <c r="A147" s="13" t="s">
         <v>717</v>
       </c>
     </row>
-    <row r="147" spans="1:1">
-      <c r="A147" s="14" t="s">
+    <row r="148" spans="1:1">
+      <c r="A148" s="13" t="s">
         <v>718</v>
       </c>
     </row>
-    <row r="148" spans="1:1">
-      <c r="A148" s="14" t="s">
+    <row r="149" spans="1:1">
+      <c r="A149" s="13" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="149" spans="1:1">
-      <c r="A149" s="14" t="s">
+    <row r="150" spans="1:1">
+      <c r="A150" s="13" t="s">
         <v>720</v>
       </c>
     </row>
-    <row r="150" spans="1:1">
-      <c r="A150" s="14" t="s">
+    <row r="151" spans="1:1">
+      <c r="A151" s="13" t="s">
         <v>721</v>
       </c>
     </row>
-    <row r="151" spans="1:1">
-      <c r="A151" s="14" t="s">
+    <row r="152" spans="1:1">
+      <c r="A152" s="13" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="152" spans="1:1">
-      <c r="A152" s="14" t="s">
+    <row r="153" spans="1:1" ht="30">
+      <c r="A153" s="13" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="153" spans="1:1" ht="30">
-      <c r="A153" s="14" t="s">
+    <row r="154" spans="1:1">
+      <c r="A154" s="13" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="154" spans="1:1">
-      <c r="A154" s="14" t="s">
+    <row r="155" spans="1:1">
+      <c r="A155" s="13" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="155" spans="1:1">
-      <c r="A155" s="14" t="s">
+    <row r="156" spans="1:1">
+      <c r="A156" s="13" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="156" spans="1:1">
-      <c r="A156" s="14" t="s">
+    <row r="157" spans="1:1">
+      <c r="A157" s="13" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="157" spans="1:1">
-      <c r="A157" s="14" t="s">
+    <row r="158" spans="1:1" ht="30">
+      <c r="A158" s="13" t="s">
         <v>728</v>
       </c>
     </row>
-    <row r="158" spans="1:1" ht="30">
-      <c r="A158" s="14" t="s">
+    <row r="159" spans="1:1">
+      <c r="A159" s="13" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="159" spans="1:1">
-      <c r="A159" s="14" t="s">
+    <row r="160" spans="1:1">
+      <c r="A160" s="13" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="160" spans="1:1">
-      <c r="A160" s="14" t="s">
+    <row r="161" spans="1:1" ht="30">
+      <c r="A161" s="13" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="161" spans="1:1" ht="30">
-      <c r="A161" s="14" t="s">
+    <row r="162" spans="1:1">
+      <c r="A162" s="13" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="162" spans="1:1">
-      <c r="A162" s="14" t="s">
+    <row r="163" spans="1:1">
+      <c r="A163" s="13" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="163" spans="1:1">
-      <c r="A163" s="14" t="s">
+    <row r="164" spans="1:1">
+      <c r="A164" s="13" t="s">
         <v>734</v>
       </c>
     </row>
-    <row r="164" spans="1:1">
-      <c r="A164" s="14" t="s">
+    <row r="165" spans="1:1">
+      <c r="A165" s="13" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="165" spans="1:1">
-      <c r="A165" s="14" t="s">
+    <row r="166" spans="1:1">
+      <c r="A166" s="13" t="s">
         <v>736</v>
       </c>
     </row>
-    <row r="166" spans="1:1">
-      <c r="A166" s="14" t="s">
+    <row r="167" spans="1:1" ht="30">
+      <c r="A167" s="13" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="167" spans="1:1" ht="30">
-      <c r="A167" s="14" t="s">
+    <row r="168" spans="1:1">
+      <c r="A168" s="13" t="s">
         <v>738</v>
       </c>
     </row>
-    <row r="168" spans="1:1">
-      <c r="A168" s="14" t="s">
+    <row r="169" spans="1:1">
+      <c r="A169" s="13" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="169" spans="1:1">
-      <c r="A169" s="14" t="s">
+    <row r="170" spans="1:1">
+      <c r="A170" s="13" t="s">
         <v>740</v>
       </c>
     </row>
-    <row r="170" spans="1:1">
-      <c r="A170" s="14" t="s">
+    <row r="171" spans="1:1" ht="30">
+      <c r="A171" s="13" t="s">
         <v>741</v>
       </c>
     </row>
-    <row r="171" spans="1:1" ht="30">
-      <c r="A171" s="14" t="s">
+    <row r="172" spans="1:1">
+      <c r="A172" s="13" t="s">
         <v>742</v>
       </c>
     </row>
-    <row r="172" spans="1:1">
-      <c r="A172" s="14" t="s">
+    <row r="173" spans="1:1">
+      <c r="A173" s="13" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="173" spans="1:1">
-      <c r="A173" s="14" t="s">
+    <row r="174" spans="1:1">
+      <c r="A174" s="13" t="s">
         <v>744</v>
       </c>
     </row>
-    <row r="174" spans="1:1">
-      <c r="A174" s="14" t="s">
+    <row r="175" spans="1:1">
+      <c r="A175" s="13" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="175" spans="1:1">
-      <c r="A175" s="14" t="s">
+    <row r="176" spans="1:1">
+      <c r="A176" s="13" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="176" spans="1:1">
-      <c r="A176" s="14" t="s">
+    <row r="177" spans="1:1">
+      <c r="A177" s="13" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="177" spans="1:1">
-      <c r="A177" s="14" t="s">
+    <row r="178" spans="1:1">
+      <c r="A178" s="13" t="s">
         <v>748</v>
       </c>
     </row>
-    <row r="178" spans="1:1">
-      <c r="A178" s="14" t="s">
+    <row r="179" spans="1:1">
+      <c r="A179" s="13" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="179" spans="1:1">
-      <c r="A179" s="14" t="s">
+    <row r="180" spans="1:1">
+      <c r="A180" s="13" t="s">
         <v>750</v>
       </c>
     </row>
-    <row r="180" spans="1:1">
-      <c r="A180" s="14" t="s">
+    <row r="181" spans="1:1">
+      <c r="A181" s="13" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="181" spans="1:1">
-      <c r="A181" s="14" t="s">
+    <row r="182" spans="1:1">
+      <c r="A182" s="13" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="182" spans="1:1">
-      <c r="A182" s="14" t="s">
+    <row r="183" spans="1:1">
+      <c r="A183" s="13" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="183" spans="1:1">
-      <c r="A183" s="14" t="s">
+    <row r="184" spans="1:1" ht="30">
+      <c r="A184" s="13" t="s">
         <v>754</v>
       </c>
     </row>
-    <row r="184" spans="1:1" ht="30">
-      <c r="A184" s="14" t="s">
+    <row r="185" spans="1:1">
+      <c r="A185" s="13" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="185" spans="1:1">
-      <c r="A185" s="14" t="s">
+    <row r="186" spans="1:1">
+      <c r="A186" s="13" t="s">
         <v>756</v>
       </c>
     </row>
-    <row r="186" spans="1:1">
-      <c r="A186" s="14" t="s">
+    <row r="187" spans="1:1">
+      <c r="A187" s="13" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="187" spans="1:1">
-      <c r="A187" s="14" t="s">
+    <row r="188" spans="1:1" ht="30">
+      <c r="A188" s="13" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="188" spans="1:1" ht="30">
-      <c r="A188" s="14" t="s">
+    <row r="189" spans="1:1">
+      <c r="A189" s="13" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="189" spans="1:1">
-      <c r="A189" s="14" t="s">
+    <row r="190" spans="1:1">
+      <c r="A190" s="13" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="190" spans="1:1">
-      <c r="A190" s="14" t="s">
+    <row r="191" spans="1:1">
+      <c r="A191" s="13" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="191" spans="1:1">
-      <c r="A191" s="14" t="s">
+    <row r="192" spans="1:1" ht="30">
+      <c r="A192" s="13" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="192" spans="1:1" ht="30">
-      <c r="A192" s="14" t="s">
+    <row r="193" spans="1:1">
+      <c r="A193" s="13" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="193" spans="1:1">
-      <c r="A193" s="14" t="s">
+    <row r="194" spans="1:1">
+      <c r="A194" s="13" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="194" spans="1:1">
-      <c r="A194" s="14" t="s">
+    <row r="195" spans="1:1">
+      <c r="A195" s="13" t="s">
         <v>765</v>
-      </c>
-    </row>
-    <row r="195" spans="1:1">
-      <c r="A195" s="14" t="s">
-        <v>766</v>
       </c>
     </row>
   </sheetData>

</xml_diff>